<commit_message>
filled in the database
</commit_message>
<xml_diff>
--- a/Base_Data.xlsx
+++ b/Base_Data.xlsx
@@ -1,10 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27932"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F396A1B-85F5-4AFB-A9D9-FE44A4E49E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="6"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Groups" sheetId="1" r:id="rId1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="101">
   <si>
     <t>ID</t>
   </si>
@@ -144,9 +145,6 @@
     <t>1800.00</t>
   </si>
   <si>
-    <t>1400.00</t>
-  </si>
-  <si>
     <t>2000.00</t>
   </si>
   <si>
@@ -159,9 +157,6 @@
     <t>1900.00</t>
   </si>
   <si>
-    <t>1550.00</t>
-  </si>
-  <si>
     <t>Прохоров П. П.</t>
   </si>
   <si>
@@ -328,13 +323,19 @@
   </si>
   <si>
     <t>1435.50</t>
+  </si>
+  <si>
+    <t>Exam_Date</t>
+  </si>
+  <si>
+    <t>Min_Score</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -342,13 +343,33 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0F1115"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0F1115"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -363,9 +384,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -647,7 +682,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -768,7 +803,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -935,99 +970,133 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+  <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
+    <col min="3" max="3" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>33</v>
+      </c>
+      <c r="C11">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -1036,7 +1105,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1060,10 +1129,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>35</v>
+        <v>43</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1500</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -1071,10 +1140,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>36</v>
+        <v>44</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1700</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1082,10 +1151,10 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>37</v>
+        <v>45</v>
+      </c>
+      <c r="C4" s="1">
+        <v>1600</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -1093,10 +1162,10 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>38</v>
+        <v>46</v>
+      </c>
+      <c r="C5" s="1">
+        <v>1800</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -1104,10 +1173,10 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1400</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -1115,10 +1184,10 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>40</v>
+        <v>48</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2000</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -1126,10 +1195,10 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>41</v>
+        <v>49</v>
+      </c>
+      <c r="C8" s="1">
+        <v>1750</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -1137,10 +1206,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>42</v>
+        <v>50</v>
+      </c>
+      <c r="C9" s="1">
+        <v>1650</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -1148,10 +1217,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>43</v>
+        <v>51</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1900</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -1159,10 +1228,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>44</v>
+        <v>52</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1550</v>
       </c>
     </row>
   </sheetData>
@@ -1171,7 +1240,7 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1185,13 +1254,13 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D1" t="s">
         <v>55</v>
-      </c>
-      <c r="C1" t="s">
-        <v>56</v>
-      </c>
-      <c r="D1" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -1204,8 +1273,8 @@
       <c r="C2">
         <v>1</v>
       </c>
-      <c r="D2" t="s">
-        <v>37</v>
+      <c r="D2" s="3">
+        <v>1600</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -1218,8 +1287,8 @@
       <c r="C3">
         <v>3</v>
       </c>
-      <c r="D3" t="s">
-        <v>38</v>
+      <c r="D3" s="3">
+        <v>1800</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -1232,8 +1301,8 @@
       <c r="C4">
         <v>2</v>
       </c>
-      <c r="D4" t="s">
-        <v>36</v>
+      <c r="D4" s="2">
+        <v>1700</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -1246,8 +1315,8 @@
       <c r="C5">
         <v>1</v>
       </c>
-      <c r="D5" t="s">
-        <v>42</v>
+      <c r="D5" s="2">
+        <v>1650</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
@@ -1260,8 +1329,8 @@
       <c r="C6">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
-        <v>43</v>
+      <c r="D6" s="2">
+        <v>1900</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
@@ -1274,8 +1343,8 @@
       <c r="C7">
         <v>5</v>
       </c>
-      <c r="D7" t="s">
-        <v>40</v>
+      <c r="D7" s="2">
+        <v>2000</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -1288,8 +1357,8 @@
       <c r="C8">
         <v>6</v>
       </c>
-      <c r="D8" t="s">
-        <v>35</v>
+      <c r="D8" s="2">
+        <v>1500</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -1302,8 +1371,8 @@
       <c r="C9">
         <v>7</v>
       </c>
-      <c r="D9" t="s">
-        <v>58</v>
+      <c r="D9" s="2">
+        <v>2100</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -1316,8 +1385,8 @@
       <c r="C10">
         <v>8</v>
       </c>
-      <c r="D10" t="s">
-        <v>59</v>
+      <c r="D10" s="2">
+        <v>1850</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
@@ -1330,8 +1399,8 @@
       <c r="C11">
         <v>9</v>
       </c>
-      <c r="D11" t="s">
-        <v>41</v>
+      <c r="D11" s="2">
+        <v>1750</v>
       </c>
     </row>
   </sheetData>
@@ -1340,202 +1409,244 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="14.85546875" customWidth="1"/>
     <col min="3" max="3" width="13.28515625" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="14.140625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="8" max="8" width="15.5703125" customWidth="1"/>
+    <col min="10" max="10" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="15.5703125" customWidth="1"/>
+    <col min="14" max="14" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C1" t="s">
+        <v>99</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>1</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
-      <c r="C2" s="1">
-        <v>1</v>
+      <c r="C2" s="5">
+        <v>46170</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>2</v>
       </c>
       <c r="B3" s="1">
         <v>2</v>
       </c>
-      <c r="C3" s="1">
-        <v>2</v>
+      <c r="C3" s="5">
+        <v>46172</v>
       </c>
       <c r="D3" s="1">
         <v>2</v>
       </c>
       <c r="E3" s="1">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+      <c r="F3">
+        <v>65</v>
+      </c>
+      <c r="J3" s="6"/>
+    </row>
+    <row r="4" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
       <c r="B4" s="1">
         <v>3</v>
       </c>
-      <c r="C4" s="1">
-        <v>3</v>
+      <c r="C4" s="5">
+        <v>46174</v>
       </c>
       <c r="D4" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E4" s="1">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+      <c r="F4">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
       <c r="B5" s="1">
         <v>4</v>
       </c>
-      <c r="C5" s="1">
+      <c r="C5" s="5">
+        <v>46176</v>
+      </c>
+      <c r="D5" s="1">
         <v>4</v>
       </c>
-      <c r="D5" s="1">
+      <c r="E5" s="1">
         <v>5</v>
       </c>
-      <c r="E5" s="1">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
       <c r="B6" s="1">
         <v>5</v>
       </c>
-      <c r="C6" s="1">
+      <c r="C6" s="5">
+        <v>46178</v>
+      </c>
+      <c r="D6" s="1">
         <v>5</v>
       </c>
-      <c r="D6" s="1">
+      <c r="E6" s="1">
         <v>4</v>
       </c>
-      <c r="E6" s="1">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
       <c r="B7" s="1">
         <v>6</v>
       </c>
-      <c r="C7" s="1">
+      <c r="C7" s="5">
+        <v>46180</v>
+      </c>
+      <c r="D7" s="1">
         <v>6</v>
       </c>
-      <c r="D7" s="1">
+      <c r="E7" s="1">
         <v>7</v>
       </c>
-      <c r="E7" s="1">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
       <c r="B8" s="1">
         <v>7</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="5">
+        <v>46182</v>
+      </c>
+      <c r="D8" s="1">
         <v>7</v>
       </c>
-      <c r="D8" s="1">
+      <c r="E8" s="1">
         <v>6</v>
       </c>
-      <c r="E8" s="1">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1">
         <v>8</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="5">
+        <v>46184</v>
+      </c>
+      <c r="D9" s="1">
         <v>8</v>
       </c>
-      <c r="D9" s="1">
+      <c r="E9" s="1">
         <v>9</v>
       </c>
-      <c r="E9" s="1">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
       <c r="B10" s="1">
         <v>9</v>
       </c>
-      <c r="C10" s="1">
+      <c r="C10" s="5">
+        <v>46186</v>
+      </c>
+      <c r="D10" s="1">
         <v>9</v>
       </c>
-      <c r="D10" s="1">
+      <c r="E10" s="1">
         <v>10</v>
       </c>
-      <c r="E10" s="1">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
       <c r="B11" s="1">
         <v>10</v>
       </c>
-      <c r="C11" s="1">
+      <c r="C11" s="5">
+        <v>46188</v>
+      </c>
+      <c r="D11" s="1">
         <v>10</v>
       </c>
-      <c r="D11" s="1">
-        <v>3</v>
-      </c>
       <c r="E11" s="1">
-        <v>90</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="F11">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8" ht="16.5" x14ac:dyDescent="0.25">
+      <c r="H21" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1543,7 +1654,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1555,6 +1666,7 @@
     <col min="6" max="6" width="17.42578125" customWidth="1"/>
     <col min="7" max="7" width="13.28515625" customWidth="1"/>
     <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="20" max="20" width="12.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1562,28 +1674,28 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>1</v>
       </c>
@@ -1597,19 +1709,19 @@
         <v>37</v>
       </c>
       <c r="E2" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="F2" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="H2" s="1">
+      <c r="H2" s="7">
         <v>45458</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2</v>
       </c>
@@ -1623,19 +1735,19 @@
         <v>36</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F3" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="H3" s="1">
+      <c r="H3" s="5">
         <v>45459</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -1649,19 +1761,19 @@
         <v>38</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="1">
+      <c r="H4" s="5">
         <v>45460</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
@@ -1672,22 +1784,22 @@
         <v>5</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E5" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="F5" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="H5" s="1">
+      <c r="H5" s="5">
         <v>45461</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
@@ -1698,22 +1810,22 @@
         <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="H6" s="1">
+      <c r="H6" s="5">
         <v>45462</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -1727,19 +1839,19 @@
         <v>35</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="H7" s="1">
+      <c r="H7" s="5">
         <v>45463</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
@@ -1750,22 +1862,22 @@
         <v>8</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H8" s="1">
+      <c r="H8" s="5">
         <v>45464</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
@@ -1776,22 +1888,22 @@
         <v>9</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="H9" s="1">
+      <c r="H9" s="5">
         <v>45465</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
@@ -1802,22 +1914,22 @@
         <v>10</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="E10" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="G10" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H10" s="1">
+      <c r="H10" s="5">
         <v>45466</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
@@ -1828,18 +1940,18 @@
         <v>4</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="G11" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="H11" s="1">
+      <c r="H11" s="5">
         <v>45467</v>
       </c>
     </row>

</xml_diff>